<commit_message>
Update editor levels and level workflow
</commit_message>
<xml_diff>
--- a/excel/关卡表.xlsx
+++ b/excel/关卡表.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\曹天宇\Desktop\NCweb\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Agent\nc2\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9247F9B-F4F2-40FC-AA71-F46F971CF4A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CC87E26-1E25-4930-9C81-528D9607A9E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,129 +16,219 @@
     <sheet name="关卡" sheetId="1" r:id="rId1"/>
     <sheet name="阵型" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="33">
   <si>
     <t>id</t>
+  </si>
+  <si>
+    <t>data</t>
+  </si>
+  <si>
+    <t>[[24,23,21,20,19],[27,25,22,18,13],[26,28,17,14,12],[1,29,15,16,11],[2,30,31,7,10],[3,32,6,9,8],[4,5,33,34,35]]</t>
+  </si>
+  <si>
+    <t>[[29,30,31,32,33],[28,26,4,3,34],[27,25,5,2,35],[23,24,6,1,36],[22,21,7,38,37],[18,20,8,40,39],[17,19,9,13,12],[16,15,14,10,11]]</t>
+  </si>
+  <si>
+    <t>[[34,36,38,42,43,44],[35,33,37,39,41,45],[31,32,29,2,40,46],[24,30,28,3,1,47],[23,25,27,4,5,48],[22,21,26,14,6,8],[20,16,15,13,7,9],[19,18,17,12,11,10]]</t>
+  </si>
+  <si>
+    <t>[[2,25,26,27,29,31],[1,3,24,28,30,32],[53,54,4,23,33,34],[50,52,6,5,22,35],[49,51,7,21,37,36],[46,48,8,38,20,19],[45,47,39,9,17,18],[44,40,41,16,10,11],[43,42,15,14,13,12]]</t>
+  </si>
+  <si>
+    <t>[[20,19,18,17,1,3],[22,21,26,16,2,4],[23,25,15,27,30,5],[24,14,11,29,28,6],[13,12,10,9,8,7]]</t>
+  </si>
+  <si>
+    <t>[[3,1,30,31,33,34],[4,2,29,28,32,35],[5,6,7,27,37,36],[22,21,26,8,39,38],[23,25,20,40,9,10],[24,19,15,41,13,11],[18,17,16,14,42,12]]</t>
+  </si>
+  <si>
+    <t>[[26,27,28,29,1,2],[24,25,32,30,3,4],[23,21,31,33,38,5],[22,20,34,37,6,39],[48,19,36,35,40,7],[47,46,18,42,41,8],[16,17,45,44,43,9],[15,14,13,12,11,10]]</t>
+  </si>
+  <si>
+    <t>[[12,11,10,16,22,21],[13,9,15,23,17,20],[8,14,24,18,19,29],[7,25,26,27,28,30],[6,3,36,1,32,31],[4,5,2,35,34,33]]</t>
+  </si>
+  <si>
+    <t>[[1,2,3,4]]</t>
+  </si>
+  <si>
+    <t>[[1,-2,3],[6,5,4],[-7,8,9]]</t>
+  </si>
+  <si>
+    <t>[[1,2,-6],[-3,5,7],[4,-8,11],[-9,10,12]]</t>
+  </si>
+  <si>
+    <t>[[1,15,16,7],[2,14,-6,8],[-3,5,-13,9],[4,12,11,-10]]</t>
+  </si>
+  <si>
+    <t>[[0,0,3,0,0],[0,2,-7,-4,0],[1,-8,9,6,5]]</t>
+  </si>
+  <si>
+    <t>[[-16,-17,18,19,-21],[15,14,-13,-22,20],[6,7,23,12,-11],[-5,24,-8,9,10],[25,4,3,-2,1]]</t>
+  </si>
+  <si>
+    <t>[[1,3,-4,5,6],[-2,24,-23,22,-7],[25,10,9,-8,21],[30,26,-11,18,20],[29,-27,17,12,-19],[28,-16,15,-14,13]]</t>
+  </si>
+  <si>
+    <t>[[-25,29,-30,31,4,-5],[-24,26,28,32,6,-3],[0,23,-27,-7,2,0],[0,19,22,1,8,0],[18,-20,21,14,-13,9],[-17,16,15,12,11,-10]]</t>
+  </si>
+  <si>
+    <t>[[1,-10,11,-13],[2,9,-14,12],[3,-15,8,-7],[16,4,-5,6]]</t>
+  </si>
+  <si>
+    <t>[[1,-2,13,-14,15],[-11,12,-3,7,-6],[10,-9,8,-4,5]]</t>
+  </si>
+  <si>
+    <t>[[-11,12,-13,-19,20],[-10,14,18,17,-21],[3,-9,-15,16,22],[-4,2,8,-7,23],[1,5,-6,25,-24]]</t>
+  </si>
+  <si>
+    <t>[[-22,-24,25,26,-28,29],[23,21,-16,27,-31,-30],[-20,15,17,-32,0,0],[19,-18,-14,33,34,-35],[0,0,12,-13,1,36],[9,10,-11,-4,2,37],[-8,7,6,5,3,38]]</t>
+  </si>
+  <si>
+    <t>[[1,13,-12],[-14,2,11],[-15,10,-3],[16,-4,9],[5,17,-8],[6,-7,18]]</t>
+  </si>
+  <si>
+    <t>[[1,-2,3,4],[-12,11,-10,5],[13,-14,9,-6],[16,15,-8,7]]</t>
+  </si>
+  <si>
+    <t>[[0,28,-29,-30,-31],[27,23,21,34,32],[-26,24,-22,20,33],[1,-25,0,0,-19],[2,0,0,-18,17],[3,-10,9,16,15],[-4,-8,11,-14,13],[5,6,-7,-12,0]]</t>
+  </si>
+  <si>
+    <t>[[-34,-35,36,-37,42,41],[33,26,-24,23,38,-40],[-32,27,25,8,22,39],[-31,29,-28,-7,9,-21],[1,-30,6,-15,20,10],[-2,5,16,19,14,-11],[-3,4,18,-17,12,-13]]</t>
+  </si>
+  <si>
+    <t>[[-36,35,34,33,27,-26,-25],[37,38,-32,30,-28,23,-24],[-40,-39,31,-44,29,22,21],[41,42,43,45,18,-19,-20],[1,47,-46,16,-17,13,12],[2,49,48,-15,14,-9,-11],[3,-4,-5,-6,7,-8,10]]</t>
+  </si>
+  <si>
+    <t>[[13,12,11,-6,7,1,2],[-14,-10,9,8,-5,-4,3],[-15,17,0,-21,0,-24,-25],[45,-16,18,-20,22,23,26],[46,-44,42,19,-29,-28,27],[-47,43,0,41,0,30,31],[48,52,38,39,-40,-34,-32],[49,50,-51,-37,36,35,-33]]</t>
+  </si>
+  <si>
+    <r>
+      <t>[1,2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>,3,4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
+      <t>]</t>
+    </r>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>data</t>
+    <r>
+      <t>[9,10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>,11,12</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
+      <t>]</t>
+    </r>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>[[1,2,3,4]]</t>
-  </si>
-  <si>
-    <t>[[1,-2,3],[6,5,4],[-7,8,9]]</t>
-  </si>
-  <si>
-    <t>[[3,4,5],[2,1,6],[9,8,7]]</t>
-  </si>
-  <si>
-    <t>[[4,5,6,7],[14,3,16,8],[13,15,2,9],[12,11,10,1]]</t>
-  </si>
-  <si>
-    <t>[[20,19,18,17,8],[21,25,16,9,7],[22,24,10,15,6],[23,11,14,5,2],[12,13,4,3,1]]</t>
-  </si>
-  <si>
-    <t>[[2,3,8,5,6,35],[1,9,4,7,36,34],[10,22,21,20,19,33],[11,23,17,18,32,29],[12,16,24,31,30,28],[13,14,15,25,26,27]]</t>
-  </si>
-  <si>
-    <t>[[22,23,25,26,27,28],[21,24,11,31,30,29],[20,14,12,10,32,34],[19,15,13,9,33,35],[18,16,8,7,36,37],[17,4,5,6,39,38],[3,2,1,42,41,40]]</t>
-  </si>
-  <si>
-    <t>[[15,16,17,18,41,1],[13,14,19,42,2,40],[12,20,10,3,4,39],[21,11,28,9,5,38],[22,27,8,29,6,37],[23,26,30,7,36,34],[24,25,31,32,33,35]]</t>
-  </si>
-  <si>
-    <t>[[3,4,10,45,46,47],[2,9,5,11,44,48],[1,8,7,6,12,43],[34,38,39,40,42,13],[33,35,37,41,15,14],[32,36,27,26,25,16],[31,28,22,23,24,17],[30,29,21,20,19,18]]</t>
-  </si>
-  <si>
-    <t>[[19,20,48,46,45,44],[5,18,21,47,43,41],[6,4,17,22,42,40],[7,16,3,23,37,39],[8,15,2,24,36,38],[9,14,1,25,29,35],[10,13,26,28,34,30],[12,11,27,33,32,31]]</t>
-  </si>
-  <si>
-    <t>[[16,17,19,20,22],[15,18,9,21,23],[14,12,10,8,24],[13,29,11,25,7],[30,28,26,4,6],[31,27,35,3,5],[32,33,34,1,2]]</t>
-  </si>
-  <si>
-    <t>[[39,38,37,25,26],[19,40,36,24,27],[18,20,23,35,28],[17,22,21,29,34],[16,14,12,30,33],[15,11,13,31,32],[10,9,4,3,1],[8,7,6,5,2]]</t>
-  </si>
-  <si>
-    <t>[[48,17,15,13,12,1],[47,16,18,14,11,2],[46,19,37,38,10,3],[20,45,39,36,9,4],[21,44,40,35,8,5],[22,41,43,34,6,7],[23,24,42,33,32,31],[25,26,27,28,29,30]]</t>
-  </si>
-  <si>
-    <t>[[31,33,34,35,36,38],[30,32,44,43,37,39],[29,45,25,23,42,40],[46,28,26,24,22,41],[1,47,27,21,11,12],[2,48,9,10,20,13],[3,8,7,18,19,14],[4,5,6,17,16,15]]</t>
-  </si>
-  <si>
-    <t>[[8,7,6,5,4,1],[9,10,30,31,2,3],[11,34,32,29,24,25],[12,35,33,23,28,26],[13,36,17,22,19,27],[14,15,16,18,21,20]]</t>
-  </si>
-  <si>
-    <t>[[14,13,11,4,3,2],[15,12,5,10,9,1],[16,17,6,8,35,36],[19,18,7,34,38,37],[31,20,33,39,40,41],[30,32,21,26,25,42],[29,28,27,22,23,24]]</t>
-  </si>
-  <si>
-    <t>[[8,7,25,24,23,22],[6,9,27,26,20,21],[5,28,10,16,17,19],[4,29,31,11,15,18],[3,30,33,32,12,14],[2,34,45,44,43,13],[35,1,46,47,48,42],[36,37,38,39,40,41]]</t>
-  </si>
-  <si>
-    <t>[[48,47,22,19,1,2],[46,23,20,21,18,3],[45,25,24,17,12,4],[26,44,16,13,11,5],[43,27,14,15,10,6],[42,36,28,34,9,7],[41,37,35,29,33,8],[40,39,38,30,31,32]]</t>
-  </si>
-  <si>
-    <t>[[24,23,21,20,19],[27,25,22,18,13],[26,28,17,14,12],[1,29,15,16,11],[2,30,31,7,10],[3,32,6,9,8],[4,5,33,34,35]]</t>
-  </si>
-  <si>
-    <t>[[29,30,31,32,33],[28,26,4,3,34],[27,25,5,2,35],[23,24,6,1,36],[22,21,7,38,37],[18,20,8,40,39],[17,19,9,13,12],[16,15,14,10,11]]</t>
-  </si>
-  <si>
-    <t>[[34,36,38,42,43,44],[35,33,37,39,41,45],[31,32,29,2,40,46],[24,30,28,3,1,47],[23,25,27,4,5,48],[22,21,26,14,6,8],[20,16,15,13,7,9],[19,18,17,12,11,10]]</t>
-  </si>
-  <si>
-    <t>[[2,25,26,27,29,31],[1,3,24,28,30,32],[53,54,4,23,33,34],[50,52,6,5,22,35],[49,51,7,21,37,36],[46,48,8,38,20,19],[45,47,39,9,17,18],[44,40,41,16,10,11],[43,42,15,14,13,12]]</t>
-  </si>
-  <si>
-    <t>[[20,19,18,17,1,3],[22,21,26,16,2,4],[23,25,15,27,30,5],[24,14,11,29,28,6],[13,12,10,9,8,7]]</t>
-  </si>
-  <si>
-    <t>[[3,1,30,31,33,34],[4,2,29,28,32,35],[5,6,7,27,37,36],[22,21,26,8,39,38],[23,25,20,40,9,10],[24,19,15,41,13,11],[18,17,16,14,42,12]]</t>
-  </si>
-  <si>
-    <t>[[26,27,28,29,1,2],[24,25,32,30,3,4],[23,21,31,33,38,5],[22,20,34,37,6,39],[48,19,36,35,40,7],[47,46,18,42,41,8],[16,17,45,44,43,9],[15,14,13,12,11,10]]</t>
-  </si>
-  <si>
-    <t>[[12,11,10,16,22,21],[13,9,15,23,17,20],[8,14,24,18,19,29],[7,25,26,27,28,30],[6,3,36,1,32,31],[4,5,2,35,34,33]]</t>
-  </si>
-  <si>
-    <t>[1,2]</t>
+    <r>
+      <t>[</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>17,18,19,20</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
+      <t>]</t>
+    </r>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>[3,4,5,6]</t>
+    <r>
+      <t>[</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>5,6,7,8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
+      <t>]</t>
+    </r>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>[7,8,9,10]</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[11,12,13,14]</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[15,16,17,18]</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[19,20,21,22]</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>[23,24,25,26]</t>
+    <r>
+      <t>[13,14</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>,15,16</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
+      <t>]</t>
+    </r>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -146,20 +236,30 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="等线"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="9"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="等线"/>
       <family val="3"/>
       <charset val="134"/>
-      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="2">
@@ -182,8 +282,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -244,74 +345,14 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Yu Gothic Light"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Yu Gothic"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Calibri"/>
+        <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -323,23 +364,23 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:tint val="67000"/>
                 <a:lumMod val="110000"/>
                 <a:satMod val="105000"/>
-                <a:tint val="67000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
+                <a:tint val="73000"/>
                 <a:lumMod val="105000"/>
                 <a:satMod val="103000"/>
-                <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
+                <a:tint val="81000"/>
                 <a:lumMod val="105000"/>
                 <a:satMod val="109000"/>
-                <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -349,23 +390,23 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
+                <a:tint val="94000"/>
+                <a:lumMod val="102000"/>
                 <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
+                <a:shade val="100000"/>
+                <a:lumMod val="100000"/>
                 <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
+                <a:shade val="78000"/>
                 <a:lumMod val="99000"/>
                 <a:satMod val="120000"/>
-                <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -373,26 +414,23 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="6350">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="12700">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="19050">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
@@ -427,17 +465,17 @@
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="93000"/>
-                <a:satMod val="150000"/>
                 <a:shade val="98000"/>
                 <a:lumMod val="102000"/>
+                <a:satMod val="150000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
                 <a:tint val="98000"/>
-                <a:satMod val="130000"/>
                 <a:shade val="90000"/>
                 <a:lumMod val="103000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
@@ -454,39 +492,12 @@
   </a:themeElements>
   <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
-</file>
-
-<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
-<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="350" row="4">
-    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </wetp:taskpane>
-</wetp:taskpanes>
-</file>
-
-<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
-<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{95E8E4AC-E840-4F1C-9F78-D5F96958092A}">
-  <we:reference id="wa200010215" version="2.0.0.0" store="zh-CN" storeType="OMEX"/>
-  <we:alternateReferences>
-    <we:reference id="wa200010215" version="2.0.0.0" store="" storeType="OMEX"/>
-  </we:alternateReferences>
-  <we:properties>
-    <we:property name="bps.codex_control.document_id" value="&quot;6f0fb157-b033-4829-a30a-c65e3679eac8&quot;"/>
-  </we:properties>
-  <we:bindings/>
-  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-</we:webextension>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
@@ -501,7 +512,7 @@
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>28</v>
       </c>
     </row>
@@ -509,59 +520,42 @@
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
-        <v>29</v>
+      <c r="B3" s="1" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
-        <v>30</v>
+      <c r="B4" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
-        <v>31</v>
+      <c r="B5" s="1" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="s">
-        <v>34</v>
+      <c r="B6" s="1" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8501DFAE-962F-425A-815E-638F8E20E95A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B27"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <sheetData>
@@ -578,7 +572,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -586,7 +580,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -594,7 +588,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>4</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
@@ -602,7 +596,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
@@ -610,7 +604,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
@@ -618,7 +612,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>7</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
@@ -626,7 +620,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>8</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
@@ -634,7 +628,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
@@ -642,7 +636,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
@@ -650,7 +644,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
@@ -658,7 +652,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
@@ -666,7 +660,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
@@ -674,7 +668,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
@@ -682,7 +676,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
@@ -690,7 +684,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
@@ -698,7 +692,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
@@ -706,7 +700,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
@@ -714,7 +708,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
@@ -722,7 +716,7 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>20</v>
+        <v>2</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
@@ -730,7 +724,7 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>21</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
@@ -738,7 +732,7 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>22</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
@@ -746,7 +740,7 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>23</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
@@ -754,7 +748,7 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>24</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
@@ -762,7 +756,7 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
@@ -770,7 +764,7 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>26</v>
+        <v>8</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
@@ -778,7 +772,7 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>27</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix puzzle workbook stage mapping
</commit_message>
<xml_diff>
--- a/excel/关卡表.xlsx
+++ b/excel/关卡表.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Agent\nc2\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CC87E26-1E25-4930-9C81-528D9607A9E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D548884C-C931-4251-BA13-8C4D5B08E56C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="关卡" sheetId="1" r:id="rId1"/>
@@ -56,179 +56,180 @@
     <t>[[1,2,3,4]]</t>
   </si>
   <si>
+    <t>[[1,2,-6],[-3,5,7],[4,-8,11],[-9,10,12]]</t>
+  </si>
+  <si>
+    <t>[[1,15,16,7],[2,14,-6,8],[-3,5,-13,9],[4,12,11,-10]]</t>
+  </si>
+  <si>
+    <t>[[0,0,3,0,0],[0,2,-7,-4,0],[1,-8,9,6,5]]</t>
+  </si>
+  <si>
+    <t>[[-16,-17,18,19,-21],[15,14,-13,-22,20],[6,7,23,12,-11],[-5,24,-8,9,10],[25,4,3,-2,1]]</t>
+  </si>
+  <si>
+    <t>[[1,3,-4,5,6],[-2,24,-23,22,-7],[25,10,9,-8,21],[30,26,-11,18,20],[29,-27,17,12,-19],[28,-16,15,-14,13]]</t>
+  </si>
+  <si>
+    <t>[[-25,29,-30,31,4,-5],[-24,26,28,32,6,-3],[0,23,-27,-7,2,0],[0,19,22,1,8,0],[18,-20,21,14,-13,9],[-17,16,15,12,11,-10]]</t>
+  </si>
+  <si>
+    <t>[[1,-10,11,-13],[2,9,-14,12],[3,-15,8,-7],[16,4,-5,6]]</t>
+  </si>
+  <si>
+    <t>[[1,-2,13,-14,15],[-11,12,-3,7,-6],[10,-9,8,-4,5]]</t>
+  </si>
+  <si>
+    <t>[[-11,12,-13,-19,20],[-10,14,18,17,-21],[3,-9,-15,16,22],[-4,2,8,-7,23],[1,5,-6,25,-24]]</t>
+  </si>
+  <si>
+    <t>[[-22,-24,25,26,-28,29],[23,21,-16,27,-31,-30],[-20,15,17,-32,0,0],[19,-18,-14,33,34,-35],[0,0,12,-13,1,36],[9,10,-11,-4,2,37],[-8,7,6,5,3,38]]</t>
+  </si>
+  <si>
+    <t>[[1,13,-12],[-14,2,11],[-15,10,-3],[16,-4,9],[5,17,-8],[6,-7,18]]</t>
+  </si>
+  <si>
+    <t>[[1,-2,3,4],[-12,11,-10,5],[13,-14,9,-6],[16,15,-8,7]]</t>
+  </si>
+  <si>
+    <t>[[0,28,-29,-30,-31],[27,23,21,34,32],[-26,24,-22,20,33],[1,-25,0,0,-19],[2,0,0,-18,17],[3,-10,9,16,15],[-4,-8,11,-14,13],[5,6,-7,-12,0]]</t>
+  </si>
+  <si>
+    <t>[[-34,-35,36,-37,42,41],[33,26,-24,23,38,-40],[-32,27,25,8,22,39],[-31,29,-28,-7,9,-21],[1,-30,6,-15,20,10],[-2,5,16,19,14,-11],[-3,4,18,-17,12,-13]]</t>
+  </si>
+  <si>
+    <t>[[-36,35,34,33,27,-26,-25],[37,38,-32,30,-28,23,-24],[-40,-39,31,-44,29,22,21],[41,42,43,45,18,-19,-20],[1,47,-46,16,-17,13,12],[2,49,48,-15,14,-9,-11],[3,-4,-5,-6,7,-8,10]]</t>
+  </si>
+  <si>
+    <t>[[13,12,11,-6,7,1,2],[-14,-10,9,8,-5,-4,3],[-15,17,0,-21,0,-24,-25],[45,-16,18,-20,22,23,26],[46,-44,42,19,-29,-28,27],[-47,43,0,41,0,30,31],[48,52,38,39,-40,-34,-32],[49,50,-51,-37,36,35,-33]]</t>
+  </si>
+  <si>
+    <r>
+      <t>[1,2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>,3,4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
+      <t>]</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>[9,10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>,11,12</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
+      <t>]</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>[</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>17,18,19,20</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
+      <t>]</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>[</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>5,6,7,8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
+      <t>]</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>[13,14</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>,15,16</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <charset val="134"/>
+      </rPr>
+      <t>]</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
     <t>[[1,-2,3],[6,5,4],[-7,8,9]]</t>
-  </si>
-  <si>
-    <t>[[1,2,-6],[-3,5,7],[4,-8,11],[-9,10,12]]</t>
-  </si>
-  <si>
-    <t>[[1,15,16,7],[2,14,-6,8],[-3,5,-13,9],[4,12,11,-10]]</t>
-  </si>
-  <si>
-    <t>[[0,0,3,0,0],[0,2,-7,-4,0],[1,-8,9,6,5]]</t>
-  </si>
-  <si>
-    <t>[[-16,-17,18,19,-21],[15,14,-13,-22,20],[6,7,23,12,-11],[-5,24,-8,9,10],[25,4,3,-2,1]]</t>
-  </si>
-  <si>
-    <t>[[1,3,-4,5,6],[-2,24,-23,22,-7],[25,10,9,-8,21],[30,26,-11,18,20],[29,-27,17,12,-19],[28,-16,15,-14,13]]</t>
-  </si>
-  <si>
-    <t>[[-25,29,-30,31,4,-5],[-24,26,28,32,6,-3],[0,23,-27,-7,2,0],[0,19,22,1,8,0],[18,-20,21,14,-13,9],[-17,16,15,12,11,-10]]</t>
-  </si>
-  <si>
-    <t>[[1,-10,11,-13],[2,9,-14,12],[3,-15,8,-7],[16,4,-5,6]]</t>
-  </si>
-  <si>
-    <t>[[1,-2,13,-14,15],[-11,12,-3,7,-6],[10,-9,8,-4,5]]</t>
-  </si>
-  <si>
-    <t>[[-11,12,-13,-19,20],[-10,14,18,17,-21],[3,-9,-15,16,22],[-4,2,8,-7,23],[1,5,-6,25,-24]]</t>
-  </si>
-  <si>
-    <t>[[-22,-24,25,26,-28,29],[23,21,-16,27,-31,-30],[-20,15,17,-32,0,0],[19,-18,-14,33,34,-35],[0,0,12,-13,1,36],[9,10,-11,-4,2,37],[-8,7,6,5,3,38]]</t>
-  </si>
-  <si>
-    <t>[[1,13,-12],[-14,2,11],[-15,10,-3],[16,-4,9],[5,17,-8],[6,-7,18]]</t>
-  </si>
-  <si>
-    <t>[[1,-2,3,4],[-12,11,-10,5],[13,-14,9,-6],[16,15,-8,7]]</t>
-  </si>
-  <si>
-    <t>[[0,28,-29,-30,-31],[27,23,21,34,32],[-26,24,-22,20,33],[1,-25,0,0,-19],[2,0,0,-18,17],[3,-10,9,16,15],[-4,-8,11,-14,13],[5,6,-7,-12,0]]</t>
-  </si>
-  <si>
-    <t>[[-34,-35,36,-37,42,41],[33,26,-24,23,38,-40],[-32,27,25,8,22,39],[-31,29,-28,-7,9,-21],[1,-30,6,-15,20,10],[-2,5,16,19,14,-11],[-3,4,18,-17,12,-13]]</t>
-  </si>
-  <si>
-    <t>[[-36,35,34,33,27,-26,-25],[37,38,-32,30,-28,23,-24],[-40,-39,31,-44,29,22,21],[41,42,43,45,18,-19,-20],[1,47,-46,16,-17,13,12],[2,49,48,-15,14,-9,-11],[3,-4,-5,-6,7,-8,10]]</t>
-  </si>
-  <si>
-    <t>[[13,12,11,-6,7,1,2],[-14,-10,9,8,-5,-4,3],[-15,17,0,-21,0,-24,-25],[45,-16,18,-20,22,23,26],[46,-44,42,19,-29,-28,27],[-47,43,0,41,0,30,31],[48,52,38,39,-40,-34,-32],[49,50,-51,-37,36,35,-33]]</t>
-  </si>
-  <si>
-    <r>
-      <t>[1,2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>,3,4</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <charset val="134"/>
-      </rPr>
-      <t>]</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>[9,10</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>,11,12</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <charset val="134"/>
-      </rPr>
-      <t>]</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>[</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>17,18,19,20</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <charset val="134"/>
-      </rPr>
-      <t>]</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>[</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>5,6,7,8</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <charset val="134"/>
-      </rPr>
-      <t>]</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>[13,14</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>,15,16</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <charset val="134"/>
-      </rPr>
-      <t>]</t>
-    </r>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -282,9 +283,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -513,7 +515,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
@@ -521,7 +523,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -529,7 +531,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
@@ -537,7 +539,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
@@ -545,7 +547,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -579,8 +581,8 @@
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
-        <v>11</v>
+      <c r="B3" s="2" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -588,7 +590,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
@@ -596,7 +598,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
@@ -604,7 +606,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
@@ -612,7 +614,7 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
@@ -620,7 +622,7 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
@@ -628,7 +630,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
@@ -636,7 +638,7 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
@@ -644,7 +646,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
@@ -652,7 +654,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
@@ -660,7 +662,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
@@ -668,7 +670,7 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
@@ -676,7 +678,7 @@
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
@@ -684,7 +686,7 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
@@ -692,7 +694,7 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
@@ -700,7 +702,7 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
@@ -708,7 +710,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">

</xml_diff>